<commit_message>
cn-#23 Adding a testing case to NOTE: Custom formatted DateTime is treated as number at this point
</commit_message>
<xml_diff>
--- a/test/Cactus.ClosedXMLNUnitTest/TestExcelFile.xlsx
+++ b/test/Cactus.ClosedXMLNUnitTest/TestExcelFile.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\itu\Cactus.net\test\Cactus.MiniExcelNUnitTest\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\itu\Cactus.net\test\Cactus.ClosedXMLNUnitTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A27EFF-A97C-4290-A458-33E4C11CDD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D282EA-5B44-4FC8-BD52-A924C90F02CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{0BED3855-2AA3-43F5-AEF6-4AF9E20534DC}"/>
+    <workbookView xWindow="29970" yWindow="375" windowWidth="28800" windowHeight="15285" activeTab="2" xr2:uid="{0BED3855-2AA3-43F5-AEF6-4AF9E20534DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="DateTime" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateCount="250" iterateDelta="1.0000000000000001E-5"/>
   <extLst>
@@ -36,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">Test </t>
   </si>
@@ -55,12 +78,18 @@
   </si>
   <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>#Not able to distinct custom formated DateTime at this point, need reformate the spredshee first to process</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="[$-409]mmm\-yy;@"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -90,8 +119,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,9 +461,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14D70C0E-043D-4029-A314-1118ED6D850F}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -437,7 +471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -453,9 +487,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE97F681-FB8A-485C-8AC6-2440CA3A95B5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -463,12 +497,65 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1C7D566-A2A2-46A6-ADFD-FD4CD3A435D3}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1">
+        <v>46207</v>
+      </c>
+      <c r="B1" t="str" cm="1">
+        <f t="array" aca="1" ref="B1" ca="1">CELL("format",A1)</f>
+        <v>D4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46204</v>
+      </c>
+      <c r="B2" t="str" cm="1">
+        <f t="array" aca="1" ref="B2" ca="1">CELL("format",A2)</f>
+        <v>D4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>46204</v>
+      </c>
+      <c r="B3" t="str" cm="1">
+        <f t="array" aca="1" ref="B3" ca="1">CELL("format",A3)</f>
+        <v>D1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B4" t="str" cm="1">
+        <f t="array" aca="1" ref="B4" ca="1">CELL("format",A4)</f>
+        <v>D3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cn-#23 To keep scientific notation for large numbers.
</commit_message>
<xml_diff>
--- a/test/Cactus.ClosedXMLNUnitTest/TestExcelFile.xlsx
+++ b/test/Cactus.ClosedXMLNUnitTest/TestExcelFile.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\itu\Cactus.net\test\Cactus.ClosedXMLNUnitTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D282EA-5B44-4FC8-BD52-A924C90F02CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9522BBDF-92B5-49F6-84F9-8FC4036D4AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29970" yWindow="375" windowWidth="28800" windowHeight="15285" activeTab="2" xr2:uid="{0BED3855-2AA3-43F5-AEF6-4AF9E20534DC}"/>
+    <workbookView xWindow="-28920" yWindow="2445" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0BED3855-2AA3-43F5-AEF6-4AF9E20534DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="DateTime" sheetId="3" r:id="rId3"/>
+    <sheet name="Number" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateCount="250" iterateDelta="1.0000000000000001E-5"/>
   <extLst>
@@ -80,7 +81,7 @@
     <t>S</t>
   </si>
   <si>
-    <t>#Not able to distinct custom formated DateTime at this point, need reformate the spredshee first to process</t>
+    <t>#Not able to distinct custom formatted DateTime at this point, need reformate the spredshee first to process</t>
   </si>
 </sst>
 </file>
@@ -88,7 +89,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-409]mmm\-yy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -119,13 +120,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,4 +563,19 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD51F285-19B7-460B-9857-5F48FBFDADCC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4">
+        <v>6.7511432520625406E-5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
cn-#23 Handle the case that ClosedXML could throw OverflowException when trying to get formatted string for 0E0
</commit_message>
<xml_diff>
--- a/test/Cactus.ClosedXMLNUnitTest/TestExcelFile.xlsx
+++ b/test/Cactus.ClosedXMLNUnitTest/TestExcelFile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\itu\Cactus.net\test\Cactus.ClosedXMLNUnitTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9522BBDF-92B5-49F6-84F9-8FC4036D4AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10820E51-6E3C-47F7-9B52-FA29D7D3E1C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2445" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0BED3855-2AA3-43F5-AEF6-4AF9E20534DC}"/>
+    <workbookView xWindow="-28920" yWindow="2445" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0BED3855-2AA3-43F5-AEF6-4AF9E20534DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">Test </t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>#Not able to distinct custom formatted DateTime at this point, need reformate the spredshee first to process</t>
+  </si>
+  <si>
+    <t>cell.GetFormattedString() will throw exception "egating the minimum value of a twos complement number is invalid"</t>
+  </si>
+  <si>
+    <t>low accuracy  number still returns float</t>
   </si>
 </sst>
 </file>
@@ -91,13 +97,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -120,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -128,6 +140,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,12 +582,33 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD51F285-19B7-460B-9857-5F48FBFDADCC}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="4">
         <v>6.7511432520625406E-5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>0.17138999999999999</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>1.4959787071234501E+18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>